<commit_message>
upload extra material for week 4
</commit_message>
<xml_diff>
--- a/wk4/Tree Inventory Data Exercise.xlsx
+++ b/wk4/Tree Inventory Data Exercise.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
-  <workbookPr codeName="ThisWorkbook" hidePivotFieldList="1"/>
+  <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Laptop W11\working_folder\Personales\Upright\Data_Science\Instructor_material\inst-dab-sep-26\wk4\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Laptop W11\working_folder\Personales\Upright\Data_Science\instructor-dab-sep-2026\wk4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C904FFE-DCA7-4267-B828-1F410B34B80A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27936A55-3514-4B47-A771-6EEED62ACD6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{422E36C7-441B-4CF8-9E4B-F37F4293F8CF}"/>
   </bookViews>
@@ -443,10 +443,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="m/d/yy\ h:mm;@"/>
-  </numFmts>
-  <fonts count="7">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -464,25 +461,6 @@
     </font>
     <font>
       <b/>
-      <sz val="8"/>
-      <color rgb="FF000000"/>
-      <name val="Helvetica Neue"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="8"/>
-      <color rgb="FF000000"/>
-      <name val="Helvetica Neue"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color theme="1"/>
-      <name val="Helvetica"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
       <sz val="14"/>
       <color theme="1"/>
       <name val="Century Gothic"/>
@@ -496,6 +474,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Century Gothic"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -505,7 +489,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -522,77 +506,15 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Heading 1 2" xfId="1" xr:uid="{78F2CDC0-5A06-4236-BE4B-C8FFA046B446}"/>
@@ -693,15 +615,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>647700</xdr:colOff>
+      <xdr:colOff>15240</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>3809</xdr:rowOff>
+      <xdr:rowOff>11429</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>22</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:colOff>38100</xdr:colOff>
       <xdr:row>75</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>7620</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -716,8 +638,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="12515850" y="175259"/>
-          <a:ext cx="8020050" cy="12807316"/>
+          <a:off x="11879580" y="186689"/>
+          <a:ext cx="8740140" cy="13087351"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2175,7 +2097,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A26C3F3F-BC28-4604-8E9D-E5F12D9EB475}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:H50"/>
-  <sheetFormatPr defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.09765625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.3984375" bestFit="1" customWidth="1"/>
@@ -2187,1304 +2109,1299 @@
     <col min="8" max="8" width="20.09765625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8">
-      <c r="A2" s="3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2">
         <v>230120</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="6">
+      <c r="D2">
         <v>5</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="F2" t="s">
         <v>11</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="G2" t="s">
         <v>9</v>
       </c>
-      <c r="H2" s="7">
+      <c r="H2">
         <v>42251.620833333334</v>
       </c>
     </row>
-    <row r="3" spans="1:8">
-      <c r="A3" s="3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3">
         <v>555509</v>
       </c>
-      <c r="B3" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C3" s="5" t="s">
+      <c r="B3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="6">
+      <c r="D3">
         <v>6</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" t="s">
         <v>14</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="F3" t="s">
         <v>15</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="G3" t="s">
         <v>16</v>
       </c>
-      <c r="H3" s="7">
+      <c r="H3">
         <v>42241.622916666667</v>
       </c>
     </row>
-    <row r="4" spans="1:8">
-      <c r="A4" s="3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4">
         <v>746627</v>
       </c>
-      <c r="B4" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" s="5" t="s">
+      <c r="B4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" t="s">
         <v>17</v>
       </c>
-      <c r="D4" s="6">
+      <c r="D4">
         <v>1</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" t="s">
         <v>18</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="F4" t="s">
         <v>19</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="G4" t="s">
         <v>20</v>
       </c>
-      <c r="H4" s="7">
+      <c r="H4">
         <v>42251.620833333334</v>
       </c>
     </row>
-    <row r="5" spans="1:8">
-      <c r="A5" s="3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5">
         <v>1058379</v>
       </c>
-      <c r="B5" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" s="5" t="s">
+      <c r="B5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" t="s">
         <v>17</v>
       </c>
-      <c r="D5" s="5">
+      <c r="D5">
         <v>1</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" t="s">
         <v>21</v>
       </c>
-      <c r="F5" s="5" t="s">
+      <c r="F5" t="s">
         <v>22</v>
       </c>
-      <c r="G5" s="5" t="s">
+      <c r="G5" t="s">
         <v>23</v>
       </c>
-      <c r="H5" s="7">
+      <c r="H5">
         <v>42278.587696759256</v>
       </c>
     </row>
-    <row r="6" spans="1:8">
-      <c r="A6" s="3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6">
         <v>1394983</v>
       </c>
-      <c r="B6" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C6" s="5" t="s">
+      <c r="B6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" t="s">
         <v>17</v>
       </c>
-      <c r="D6" s="5">
+      <c r="D6">
         <v>1</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="E6" t="s">
         <v>24</v>
       </c>
-      <c r="F6" s="5" t="s">
+      <c r="F6" t="s">
         <v>25</v>
       </c>
-      <c r="G6" s="5" t="s">
+      <c r="G6" t="s">
         <v>20</v>
       </c>
-      <c r="H6" s="7">
+      <c r="H6">
         <v>42306.527418981481</v>
       </c>
     </row>
-    <row r="7" spans="1:8">
-      <c r="A7" s="3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7">
         <v>1390660</v>
       </c>
-      <c r="B7" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C7" s="5" t="s">
+      <c r="B7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" t="s">
         <v>17</v>
       </c>
-      <c r="D7" s="5"/>
-      <c r="E7" s="5" t="s">
+      <c r="E7" t="s">
         <v>26</v>
       </c>
-      <c r="F7" s="5" t="s">
+      <c r="F7" t="s">
         <v>27</v>
       </c>
-      <c r="G7" s="5" t="s">
+      <c r="G7" t="s">
         <v>28</v>
       </c>
-      <c r="H7" s="7">
+      <c r="H7">
         <v>42306.516817129632</v>
       </c>
     </row>
-    <row r="8" spans="1:8">
-      <c r="A8" s="3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8">
         <v>1411921</v>
       </c>
-      <c r="B8" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C8" s="5" t="s">
+      <c r="B8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" t="s">
         <v>29</v>
       </c>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5" t="s">
+      <c r="E8" t="s">
         <v>30</v>
       </c>
-      <c r="F8" s="5" t="s">
+      <c r="F8" t="s">
         <v>31</v>
       </c>
-      <c r="G8" s="5" t="s">
+      <c r="G8" t="s">
         <v>9</v>
       </c>
-      <c r="H8" s="7">
+      <c r="H8">
         <v>42306.568449074075</v>
       </c>
     </row>
-    <row r="9" spans="1:8">
-      <c r="A9" s="3">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9">
         <v>1453653</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" t="s">
         <v>8</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" t="s">
         <v>29</v>
       </c>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5" t="s">
+      <c r="E9" t="s">
         <v>32</v>
       </c>
-      <c r="F9" s="5" t="s">
+      <c r="F9" t="s">
         <v>33</v>
       </c>
-      <c r="G9" s="5" t="s">
+      <c r="G9" t="s">
         <v>9</v>
       </c>
-      <c r="H9" s="7">
+      <c r="H9">
         <v>42306.668819444443</v>
       </c>
     </row>
-    <row r="10" spans="1:8">
-      <c r="A10" s="3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10">
         <v>1959661</v>
       </c>
-      <c r="B10" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C10" s="5" t="s">
+      <c r="B10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C10" t="s">
         <v>17</v>
       </c>
-      <c r="D10" s="6">
+      <c r="D10">
         <v>10</v>
       </c>
-      <c r="E10" s="5" t="s">
+      <c r="E10" t="s">
         <v>34</v>
       </c>
-      <c r="F10" s="5" t="s">
+      <c r="F10" t="s">
         <v>35</v>
       </c>
-      <c r="G10" s="5" t="s">
+      <c r="G10" t="s">
         <v>20</v>
       </c>
-      <c r="H10" s="7">
+      <c r="H10">
         <v>42360.749305555553</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="23.4">
-      <c r="A11" s="3">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11">
         <v>1744792</v>
       </c>
-      <c r="B11" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C11" s="5" t="s">
+      <c r="B11" t="s">
+        <v>12</v>
+      </c>
+      <c r="C11" t="s">
         <v>9</v>
       </c>
-      <c r="D11" s="6" t="s">
+      <c r="D11" t="s">
         <v>36</v>
       </c>
-      <c r="E11" s="5" t="s">
+      <c r="E11" t="s">
         <v>37</v>
       </c>
-      <c r="F11" s="5" t="s">
+      <c r="F11" t="s">
         <v>38</v>
       </c>
-      <c r="G11" s="5" t="s">
+      <c r="G11" t="s">
         <v>9</v>
       </c>
-      <c r="H11" s="7">
+      <c r="H11">
         <v>42338.868055555555</v>
       </c>
     </row>
-    <row r="12" spans="1:8">
-      <c r="A12" s="3">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12">
         <v>2255195</v>
       </c>
-      <c r="B12" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C12" s="5" t="s">
+      <c r="B12" t="s">
+        <v>12</v>
+      </c>
+      <c r="C12" t="s">
         <v>29</v>
       </c>
-      <c r="D12" s="5">
+      <c r="D12">
         <v>13</v>
       </c>
-      <c r="E12" s="5" t="s">
+      <c r="E12" t="s">
         <v>39</v>
       </c>
-      <c r="F12" s="5" t="s">
+      <c r="F12" t="s">
         <v>40</v>
       </c>
-      <c r="G12" s="5" t="s">
+      <c r="G12" t="s">
         <v>9</v>
       </c>
-      <c r="H12" s="7">
+      <c r="H12">
         <v>42374.713368055556</v>
       </c>
     </row>
-    <row r="13" spans="1:8">
-      <c r="A13" s="3">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13">
         <v>2263267</v>
       </c>
-      <c r="B13" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C13" s="5" t="s">
+      <c r="B13" t="s">
+        <v>12</v>
+      </c>
+      <c r="C13" t="s">
         <v>13</v>
       </c>
-      <c r="D13" s="5">
+      <c r="D13">
         <v>1</v>
       </c>
-      <c r="E13" s="5" t="s">
+      <c r="E13" t="s">
         <v>41</v>
       </c>
-      <c r="F13" s="5" t="s">
+      <c r="F13" t="s">
         <v>42</v>
       </c>
-      <c r="G13" s="5" t="s">
+      <c r="G13" t="s">
         <v>43</v>
       </c>
-      <c r="H13" s="7">
+      <c r="H13">
         <v>42374.803773148145</v>
       </c>
     </row>
-    <row r="14" spans="1:8">
-      <c r="A14" s="3">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14">
         <v>2416097</v>
       </c>
-      <c r="B14" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C14" s="5" t="s">
+      <c r="B14" t="s">
+        <v>12</v>
+      </c>
+      <c r="C14" t="s">
         <v>17</v>
       </c>
-      <c r="D14" s="5">
+      <c r="D14">
         <v>23</v>
       </c>
-      <c r="E14" s="5" t="s">
+      <c r="E14" t="s">
         <v>44</v>
       </c>
-      <c r="F14" s="5" t="s">
+      <c r="F14" t="s">
         <v>45</v>
       </c>
-      <c r="G14" s="5" t="s">
+      <c r="G14" t="s">
         <v>20</v>
       </c>
-      <c r="H14" s="7">
+      <c r="H14">
         <v>42374.733229166668</v>
       </c>
     </row>
-    <row r="15" spans="1:8">
-      <c r="A15" s="3">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15">
         <v>2419844</v>
       </c>
-      <c r="B15" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C15" s="5" t="s">
+      <c r="B15" t="s">
+        <v>12</v>
+      </c>
+      <c r="C15" t="s">
         <v>29</v>
       </c>
-      <c r="D15" s="5">
+      <c r="D15">
         <v>7</v>
       </c>
-      <c r="E15" s="5" t="s">
+      <c r="E15" t="s">
         <v>46</v>
       </c>
-      <c r="F15" s="5" t="s">
+      <c r="F15" t="s">
         <v>47</v>
       </c>
-      <c r="G15" s="5" t="s">
+      <c r="G15" t="s">
         <v>9</v>
       </c>
-      <c r="H15" s="7">
+      <c r="H15">
         <v>42374.745648148149</v>
       </c>
     </row>
-    <row r="16" spans="1:8">
-      <c r="A16" s="3">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16">
         <v>2418901</v>
       </c>
-      <c r="B16" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C16" s="5" t="s">
+      <c r="B16" t="s">
+        <v>12</v>
+      </c>
+      <c r="C16" t="s">
         <v>17</v>
       </c>
-      <c r="D16" s="5">
+      <c r="D16">
         <v>20</v>
       </c>
-      <c r="E16" s="5" t="s">
+      <c r="E16" t="s">
         <v>48</v>
       </c>
-      <c r="F16" s="5" t="s">
+      <c r="F16" t="s">
         <v>49</v>
       </c>
-      <c r="G16" s="5" t="s">
+      <c r="G16" t="s">
         <v>20</v>
       </c>
-      <c r="H16" s="7">
+      <c r="H16">
         <v>42374.7425</v>
       </c>
     </row>
-    <row r="17" spans="1:8">
-      <c r="A17" s="3">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17">
         <v>2417925</v>
       </c>
-      <c r="B17" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C17" s="5" t="s">
+      <c r="B17" t="s">
+        <v>12</v>
+      </c>
+      <c r="C17" t="s">
         <v>29</v>
       </c>
-      <c r="D17" s="5">
+      <c r="D17">
         <v>21</v>
       </c>
-      <c r="E17" s="5" t="s">
+      <c r="E17" t="s">
         <v>50</v>
       </c>
-      <c r="F17" s="5" t="s">
+      <c r="F17" t="s">
         <v>51</v>
       </c>
-      <c r="G17" s="5" t="s">
+      <c r="G17" t="s">
         <v>9</v>
       </c>
-      <c r="H17" s="7">
+      <c r="H17">
         <v>42374.739212962966</v>
       </c>
     </row>
-    <row r="18" spans="1:8">
-      <c r="A18" s="3">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18">
         <v>2508137</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="B18" t="s">
         <v>52</v>
       </c>
-      <c r="C18" s="5" t="s">
+      <c r="C18" t="s">
         <v>9</v>
       </c>
-      <c r="D18" s="5">
+      <c r="D18">
         <v>6</v>
       </c>
-      <c r="E18" s="5" t="s">
+      <c r="E18" t="s">
         <v>53</v>
       </c>
-      <c r="F18" s="5" t="s">
+      <c r="F18" t="s">
         <v>54</v>
       </c>
-      <c r="G18" s="5" t="s">
+      <c r="G18" t="s">
         <v>9</v>
       </c>
-      <c r="H18" s="7">
+      <c r="H18">
         <v>42374.802997685183</v>
       </c>
     </row>
-    <row r="19" spans="1:8">
-      <c r="A19" s="3">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19">
         <v>2551937</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="B19" t="s">
         <v>8</v>
       </c>
-      <c r="C19" s="5" t="s">
+      <c r="C19" t="s">
         <v>29</v>
       </c>
-      <c r="D19" s="5">
+      <c r="D19">
         <v>15</v>
       </c>
-      <c r="E19" s="5" t="s">
+      <c r="E19" t="s">
         <v>55</v>
       </c>
-      <c r="F19" s="5" t="s">
+      <c r="F19" t="s">
         <v>56</v>
       </c>
-      <c r="G19" s="5" t="s">
+      <c r="G19" t="s">
         <v>9</v>
       </c>
-      <c r="H19" s="7">
+      <c r="H19">
         <v>42412.656504629631</v>
       </c>
     </row>
-    <row r="20" spans="1:8">
-      <c r="A20" s="3">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20">
         <v>2605467</v>
       </c>
-      <c r="B20" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C20" s="5" t="s">
+      <c r="B20" t="s">
+        <v>12</v>
+      </c>
+      <c r="C20" t="s">
         <v>17</v>
       </c>
-      <c r="D20" s="5">
+      <c r="D20">
         <v>4</v>
       </c>
-      <c r="E20" s="5" t="s">
+      <c r="E20" t="s">
         <v>57</v>
       </c>
-      <c r="F20" s="5" t="s">
+      <c r="F20" t="s">
         <v>58</v>
       </c>
-      <c r="G20" s="5" t="s">
+      <c r="G20" t="s">
         <v>59</v>
       </c>
-      <c r="H20" s="7">
+      <c r="H20">
         <v>42374.758483796293</v>
       </c>
     </row>
-    <row r="21" spans="1:8">
-      <c r="A21" s="3">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21">
         <v>2639139</v>
       </c>
-      <c r="B21" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C21" s="5" t="s">
+      <c r="B21" t="s">
+        <v>12</v>
+      </c>
+      <c r="C21" t="s">
         <v>17</v>
       </c>
-      <c r="D21" s="5">
+      <c r="D21">
         <v>23</v>
       </c>
-      <c r="E21" s="5" t="s">
+      <c r="E21" t="s">
         <v>60</v>
       </c>
-      <c r="F21" s="5" t="s">
+      <c r="F21" t="s">
         <v>61</v>
       </c>
-      <c r="G21" s="5" t="s">
+      <c r="G21" t="s">
         <v>20</v>
       </c>
-      <c r="H21" s="7">
+      <c r="H21">
         <v>42412.709918981483</v>
       </c>
     </row>
-    <row r="22" spans="1:8">
-      <c r="A22" s="3">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22">
         <v>2909204</v>
       </c>
-      <c r="B22" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C22" s="5" t="s">
+      <c r="B22" t="s">
+        <v>12</v>
+      </c>
+      <c r="C22" t="s">
         <v>62</v>
       </c>
-      <c r="D22" s="5">
+      <c r="D22">
         <v>14</v>
       </c>
-      <c r="E22" s="5" t="s">
+      <c r="E22" t="s">
         <v>63</v>
       </c>
-      <c r="F22" s="5" t="s">
+      <c r="F22" t="s">
         <v>64</v>
       </c>
-      <c r="G22" s="5" t="s">
+      <c r="G22" t="s">
         <v>20</v>
       </c>
-      <c r="H22" s="7">
+      <c r="H22">
         <v>42412.68577546296</v>
       </c>
     </row>
-    <row r="23" spans="1:8">
-      <c r="A23" s="3">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23">
         <v>2909180</v>
       </c>
-      <c r="B23" s="5" t="s">
+      <c r="B23" t="s">
         <v>52</v>
       </c>
-      <c r="C23" s="5" t="s">
+      <c r="C23" t="s">
         <v>9</v>
       </c>
-      <c r="D23" s="5">
+      <c r="D23">
         <v>11</v>
       </c>
-      <c r="E23" s="5" t="s">
+      <c r="E23" t="s">
         <v>65</v>
       </c>
-      <c r="F23" s="5" t="s">
+      <c r="F23" t="s">
         <v>66</v>
       </c>
-      <c r="G23" s="5" t="s">
+      <c r="G23" t="s">
         <v>9</v>
       </c>
-      <c r="H23" s="7">
+      <c r="H23">
         <v>42374.836643518516</v>
       </c>
     </row>
-    <row r="24" spans="1:8">
-      <c r="A24" s="3">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24">
         <v>2911733</v>
       </c>
-      <c r="B24" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C24" s="5" t="s">
+      <c r="B24" t="s">
+        <v>12</v>
+      </c>
+      <c r="C24" t="s">
         <v>17</v>
       </c>
-      <c r="D24" s="5">
+      <c r="D24">
         <v>19</v>
       </c>
-      <c r="E24" s="5" t="s">
+      <c r="E24" t="s">
         <v>67</v>
       </c>
-      <c r="F24" s="5" t="s">
+      <c r="F24" t="s">
         <v>68</v>
       </c>
-      <c r="G24" s="5" t="s">
+      <c r="G24" t="s">
         <v>43</v>
       </c>
-      <c r="H24" s="7">
+      <c r="H24">
         <v>42444.653993055559</v>
       </c>
     </row>
-    <row r="25" spans="1:8">
-      <c r="A25" s="3">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25">
         <v>2916983</v>
       </c>
-      <c r="B25" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C25" s="5" t="s">
+      <c r="B25" t="s">
+        <v>12</v>
+      </c>
+      <c r="C25" t="s">
         <v>17</v>
       </c>
-      <c r="D25" s="5">
+      <c r="D25">
         <v>9</v>
       </c>
-      <c r="E25" s="5" t="s">
+      <c r="E25" t="s">
         <v>69</v>
       </c>
-      <c r="F25" s="5" t="s">
+      <c r="F25" t="s">
         <v>70</v>
       </c>
-      <c r="G25" s="5" t="s">
+      <c r="G25" t="s">
         <v>71</v>
       </c>
-      <c r="H25" s="7">
+      <c r="H25">
         <v>42444.666585648149</v>
       </c>
     </row>
-    <row r="26" spans="1:8">
-      <c r="A26" s="3">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26">
         <v>3009624</v>
       </c>
-      <c r="B26" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C26" s="5" t="s">
+      <c r="B26" t="s">
+        <v>12</v>
+      </c>
+      <c r="C26" t="s">
         <v>9</v>
       </c>
-      <c r="D26" s="5">
+      <c r="D26">
         <v>9</v>
       </c>
-      <c r="E26" s="5" t="s">
+      <c r="E26" t="s">
         <v>72</v>
       </c>
-      <c r="F26" s="5" t="s">
+      <c r="F26" t="s">
         <v>73</v>
       </c>
-      <c r="G26" s="5" t="s">
+      <c r="G26" t="s">
         <v>9</v>
       </c>
-      <c r="H26" s="7">
+      <c r="H26">
         <v>42463.736805555556</v>
       </c>
     </row>
-    <row r="27" spans="1:8">
-      <c r="A27" s="3">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A27">
         <v>3352205</v>
       </c>
-      <c r="B27" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C27" s="5" t="s">
+      <c r="B27" t="s">
+        <v>12</v>
+      </c>
+      <c r="C27" t="s">
         <v>17</v>
       </c>
-      <c r="D27" s="5">
+      <c r="D27">
         <v>8</v>
       </c>
-      <c r="E27" s="5" t="s">
+      <c r="E27" t="s">
         <v>74</v>
       </c>
-      <c r="F27" s="5" t="s">
+      <c r="F27" t="s">
         <v>75</v>
       </c>
-      <c r="G27" s="5" t="s">
+      <c r="G27" t="s">
         <v>23</v>
       </c>
-      <c r="H27" s="7">
+      <c r="H27">
         <v>42501.743379629632</v>
       </c>
     </row>
-    <row r="28" spans="1:8">
-      <c r="A28" s="3">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A28">
         <v>3359946</v>
       </c>
-      <c r="B28" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C28" s="5" t="s">
+      <c r="B28" t="s">
+        <v>12</v>
+      </c>
+      <c r="C28" t="s">
         <v>17</v>
       </c>
-      <c r="D28" s="5">
+      <c r="D28">
         <v>14</v>
       </c>
-      <c r="E28" s="5" t="s">
+      <c r="E28" t="s">
         <v>76</v>
       </c>
-      <c r="F28" s="5" t="s">
+      <c r="F28" t="s">
         <v>77</v>
       </c>
-      <c r="G28" s="5" t="s">
+      <c r="G28" t="s">
         <v>23</v>
       </c>
-      <c r="H28" s="7">
+      <c r="H28">
         <v>42501.87226851852</v>
       </c>
     </row>
-    <row r="29" spans="1:8">
-      <c r="A29" s="3">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A29">
         <v>3648707</v>
       </c>
-      <c r="B29" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C29" s="5" t="s">
+      <c r="B29" t="s">
+        <v>12</v>
+      </c>
+      <c r="C29" t="s">
         <v>17</v>
       </c>
-      <c r="D29" s="5">
+      <c r="D29">
         <v>7</v>
       </c>
-      <c r="E29" s="5" t="s">
+      <c r="E29" t="s">
         <v>78</v>
       </c>
-      <c r="F29" s="5" t="s">
+      <c r="F29" t="s">
         <v>79</v>
       </c>
-      <c r="G29" s="5" t="s">
+      <c r="G29" t="s">
         <v>20</v>
       </c>
-      <c r="H29" s="7">
+      <c r="H29">
         <v>42501.804363425923</v>
       </c>
     </row>
-    <row r="30" spans="1:8">
-      <c r="A30" s="3">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A30">
         <v>3731604</v>
       </c>
-      <c r="B30" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C30" s="5" t="s">
+      <c r="B30" t="s">
+        <v>12</v>
+      </c>
+      <c r="C30" t="s">
         <v>17</v>
       </c>
-      <c r="D30" s="5">
+      <c r="D30">
         <v>9</v>
       </c>
-      <c r="E30" s="5" t="s">
+      <c r="E30" t="s">
         <v>80</v>
       </c>
-      <c r="F30" s="5" t="s">
+      <c r="F30" t="s">
         <v>81</v>
       </c>
-      <c r="G30" s="5" t="s">
+      <c r="G30" t="s">
         <v>71</v>
       </c>
-      <c r="H30" s="7">
+      <c r="H30">
         <v>42542.632106481484</v>
       </c>
     </row>
-    <row r="31" spans="1:8">
-      <c r="A31" s="3">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A31">
         <v>3727280</v>
       </c>
-      <c r="B31" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C31" s="5" t="s">
+      <c r="B31" t="s">
+        <v>12</v>
+      </c>
+      <c r="C31" t="s">
         <v>17</v>
       </c>
-      <c r="D31" s="5">
+      <c r="D31">
         <v>21</v>
       </c>
-      <c r="E31" s="5" t="s">
+      <c r="E31" t="s">
         <v>82</v>
       </c>
-      <c r="F31" s="5" t="s">
+      <c r="F31" t="s">
         <v>83</v>
       </c>
-      <c r="G31" s="5" t="s">
+      <c r="G31" t="s">
         <v>59</v>
       </c>
-      <c r="H31" s="7">
+      <c r="H31">
         <v>42542.608784722222</v>
       </c>
     </row>
-    <row r="32" spans="1:8">
-      <c r="A32" s="3">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A32">
         <v>3741425</v>
       </c>
-      <c r="B32" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C32" s="5" t="s">
+      <c r="B32" t="s">
+        <v>12</v>
+      </c>
+      <c r="C32" t="s">
         <v>17</v>
       </c>
-      <c r="D32" s="5">
+      <c r="D32">
         <v>19</v>
       </c>
-      <c r="E32" s="5" t="s">
+      <c r="E32" t="s">
         <v>84</v>
       </c>
-      <c r="F32" s="5" t="s">
+      <c r="F32" t="s">
         <v>85</v>
       </c>
-      <c r="G32" s="5" t="s">
+      <c r="G32" t="s">
         <v>20</v>
       </c>
-      <c r="H32" s="7">
+      <c r="H32">
         <v>42542.648865740739</v>
       </c>
     </row>
-    <row r="33" spans="1:8">
-      <c r="A33" s="3">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A33">
         <v>3749038</v>
       </c>
-      <c r="B33" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C33" s="5" t="s">
+      <c r="B33" t="s">
+        <v>12</v>
+      </c>
+      <c r="C33" t="s">
         <v>17</v>
       </c>
-      <c r="D33" s="5">
+      <c r="D33">
         <v>3</v>
       </c>
-      <c r="E33" s="5" t="s">
+      <c r="E33" t="s">
         <v>86</v>
       </c>
-      <c r="F33" s="5" t="s">
+      <c r="F33" t="s">
         <v>87</v>
       </c>
-      <c r="G33" s="5" t="s">
+      <c r="G33" t="s">
         <v>59</v>
       </c>
-      <c r="H33" s="7">
+      <c r="H33">
         <v>42542.615717592591</v>
       </c>
     </row>
-    <row r="34" spans="1:8">
-      <c r="A34" s="3">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A34">
         <v>3761737</v>
       </c>
-      <c r="B34" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C34" s="5" t="s">
+      <c r="B34" t="s">
+        <v>12</v>
+      </c>
+      <c r="C34" t="s">
         <v>17</v>
       </c>
-      <c r="D34" s="5">
+      <c r="D34">
         <v>11</v>
       </c>
-      <c r="E34" s="5" t="s">
+      <c r="E34" t="s">
         <v>88</v>
       </c>
-      <c r="F34" s="5" t="s">
+      <c r="F34" t="s">
         <v>89</v>
       </c>
-      <c r="G34" s="5" t="s">
+      <c r="G34" t="s">
         <v>59</v>
       </c>
-      <c r="H34" s="7">
+      <c r="H34">
         <v>42542.618946759256</v>
       </c>
     </row>
-    <row r="35" spans="1:8">
-      <c r="A35" s="3">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A35">
         <v>3767759</v>
       </c>
-      <c r="B35" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C35" s="5" t="s">
+      <c r="B35" t="s">
+        <v>12</v>
+      </c>
+      <c r="C35" t="s">
         <v>13</v>
       </c>
-      <c r="D35" s="5">
+      <c r="D35">
         <v>20</v>
       </c>
-      <c r="E35" s="5" t="s">
+      <c r="E35" t="s">
         <v>90</v>
       </c>
-      <c r="F35" s="5" t="s">
+      <c r="F35" t="s">
         <v>91</v>
       </c>
-      <c r="G35" s="5" t="s">
+      <c r="G35" t="s">
         <v>92</v>
       </c>
-      <c r="H35" s="7">
+      <c r="H35">
         <v>42542.66542824074</v>
       </c>
     </row>
-    <row r="36" spans="1:8">
-      <c r="A36" s="3">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A36">
         <v>3998871</v>
       </c>
-      <c r="B36" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C36" s="5" t="s">
+      <c r="B36" t="s">
+        <v>12</v>
+      </c>
+      <c r="C36" t="s">
         <v>17</v>
       </c>
-      <c r="D36" s="5">
+      <c r="D36">
         <v>14</v>
       </c>
-      <c r="E36" s="5" t="s">
+      <c r="E36" t="s">
         <v>93</v>
       </c>
-      <c r="F36" s="5" t="s">
+      <c r="F36" t="s">
         <v>94</v>
       </c>
-      <c r="G36" s="5" t="s">
+      <c r="G36" t="s">
         <v>23</v>
       </c>
-      <c r="H36" s="7">
+      <c r="H36">
         <v>42551.408032407409</v>
       </c>
     </row>
-    <row r="37" spans="1:8">
-      <c r="A37" s="3">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A37">
         <v>4005560</v>
       </c>
-      <c r="B37" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C37" s="5" t="s">
+      <c r="B37" t="s">
+        <v>12</v>
+      </c>
+      <c r="C37" t="s">
         <v>17</v>
       </c>
-      <c r="D37" s="5">
+      <c r="D37">
         <v>8</v>
       </c>
-      <c r="E37" s="5" t="s">
+      <c r="E37" t="s">
         <v>95</v>
       </c>
-      <c r="F37" s="5" t="s">
+      <c r="F37" t="s">
         <v>96</v>
       </c>
-      <c r="G37" s="5" t="s">
+      <c r="G37" t="s">
         <v>97</v>
       </c>
-      <c r="H37" s="7">
+      <c r="H37">
         <v>42551.419189814813</v>
       </c>
     </row>
-    <row r="38" spans="1:8">
-      <c r="A38" s="3">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A38">
         <v>4002704</v>
       </c>
-      <c r="B38" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C38" s="5" t="s">
+      <c r="B38" t="s">
+        <v>12</v>
+      </c>
+      <c r="C38" t="s">
         <v>17</v>
       </c>
-      <c r="D38" s="5">
+      <c r="D38">
         <v>7</v>
       </c>
-      <c r="E38" s="5" t="s">
+      <c r="E38" t="s">
         <v>98</v>
       </c>
-      <c r="F38" s="5" t="s">
+      <c r="F38" t="s">
         <v>99</v>
       </c>
-      <c r="G38" s="5" t="s">
+      <c r="G38" t="s">
         <v>16</v>
       </c>
-      <c r="H38" s="7">
+      <c r="H38">
         <v>42578.540219907409</v>
       </c>
     </row>
-    <row r="39" spans="1:8">
-      <c r="A39" s="3">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A39">
         <v>4000132</v>
       </c>
-      <c r="B39" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C39" s="5" t="s">
+      <c r="B39" t="s">
+        <v>12</v>
+      </c>
+      <c r="C39" t="s">
         <v>17</v>
       </c>
-      <c r="D39" s="5">
+      <c r="D39">
         <v>1</v>
       </c>
-      <c r="E39" s="5" t="s">
+      <c r="E39" t="s">
         <v>100</v>
       </c>
-      <c r="F39" s="5" t="s">
+      <c r="F39" t="s">
         <v>101</v>
       </c>
-      <c r="G39" s="5" t="s">
+      <c r="G39" t="s">
         <v>59</v>
       </c>
-      <c r="H39" s="7">
+      <c r="H39">
         <v>42551.427673611113</v>
       </c>
     </row>
-    <row r="40" spans="1:8">
-      <c r="A40" s="3">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A40">
         <v>4018019</v>
       </c>
-      <c r="B40" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C40" s="5" t="s">
+      <c r="B40" t="s">
+        <v>12</v>
+      </c>
+      <c r="C40" t="s">
         <v>17</v>
       </c>
-      <c r="D40" s="5">
+      <c r="D40">
         <v>1</v>
       </c>
-      <c r="E40" s="5" t="s">
+      <c r="E40" t="s">
         <v>102</v>
       </c>
-      <c r="F40" s="5" t="s">
+      <c r="F40" t="s">
         <v>103</v>
       </c>
-      <c r="G40" s="5" t="s">
+      <c r="G40" t="s">
         <v>20</v>
       </c>
-      <c r="H40" s="7">
+      <c r="H40">
         <v>42578.545856481483</v>
       </c>
     </row>
-    <row r="41" spans="1:8">
-      <c r="A41" s="3">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A41">
         <v>4020848</v>
       </c>
-      <c r="B41" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C41" s="5" t="s">
+      <c r="B41" t="s">
+        <v>12</v>
+      </c>
+      <c r="C41" t="s">
         <v>17</v>
       </c>
-      <c r="D41" s="5">
+      <c r="D41">
         <v>11</v>
       </c>
-      <c r="E41" s="5" t="s">
+      <c r="E41" t="s">
         <v>104</v>
       </c>
-      <c r="F41" s="5" t="s">
+      <c r="F41" t="s">
         <v>105</v>
       </c>
-      <c r="G41" s="5" t="s">
+      <c r="G41" t="s">
         <v>106</v>
       </c>
-      <c r="H41" s="7">
+      <c r="H41">
         <v>42551.413703703707</v>
       </c>
     </row>
-    <row r="42" spans="1:8">
-      <c r="A42" s="3">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A42">
         <v>4141883</v>
       </c>
-      <c r="B42" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C42" s="5" t="s">
+      <c r="B42" t="s">
+        <v>12</v>
+      </c>
+      <c r="C42" t="s">
         <v>17</v>
       </c>
-      <c r="D42" s="5">
+      <c r="D42">
         <v>23</v>
       </c>
-      <c r="E42" s="5" t="s">
+      <c r="E42" t="s">
         <v>107</v>
       </c>
-      <c r="F42" s="5" t="s">
+      <c r="F42" t="s">
         <v>108</v>
       </c>
-      <c r="G42" s="5" t="s">
+      <c r="G42" t="s">
         <v>16</v>
       </c>
-      <c r="H42" s="7">
+      <c r="H42">
         <v>42578.617766203701</v>
       </c>
     </row>
-    <row r="43" spans="1:8">
-      <c r="A43" s="3">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A43">
         <v>4140502</v>
       </c>
-      <c r="B43" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C43" s="5" t="s">
+      <c r="B43" t="s">
+        <v>12</v>
+      </c>
+      <c r="C43" t="s">
         <v>17</v>
       </c>
-      <c r="D43" s="5">
+      <c r="D43">
         <v>17</v>
       </c>
-      <c r="E43" s="5" t="s">
+      <c r="E43" t="s">
         <v>109</v>
       </c>
-      <c r="F43" s="5" t="s">
+      <c r="F43" t="s">
         <v>110</v>
       </c>
-      <c r="G43" s="5" t="s">
+      <c r="G43" t="s">
         <v>111</v>
       </c>
-      <c r="H43" s="7">
+      <c r="H43">
         <v>42578.649247685185</v>
       </c>
     </row>
-    <row r="44" spans="1:8">
-      <c r="A44" s="3">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A44">
         <v>4145558</v>
       </c>
-      <c r="B44" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C44" s="5" t="s">
+      <c r="B44" t="s">
+        <v>12</v>
+      </c>
+      <c r="C44" t="s">
         <v>62</v>
       </c>
-      <c r="D44" s="5">
+      <c r="D44">
         <v>22</v>
       </c>
-      <c r="E44" s="5" t="s">
+      <c r="E44" t="s">
         <v>112</v>
       </c>
-      <c r="F44" s="5" t="s">
+      <c r="F44" t="s">
         <v>113</v>
       </c>
-      <c r="G44" s="5" t="s">
+      <c r="G44" t="s">
         <v>20</v>
       </c>
-      <c r="H44" s="7">
+      <c r="H44">
         <v>42578.629953703705</v>
       </c>
     </row>
-    <row r="45" spans="1:8">
-      <c r="A45" s="3">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A45">
         <v>4145530</v>
       </c>
-      <c r="B45" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C45" s="5" t="s">
+      <c r="B45" t="s">
+        <v>12</v>
+      </c>
+      <c r="C45" t="s">
         <v>17</v>
       </c>
-      <c r="D45" s="5">
+      <c r="D45">
         <v>6</v>
       </c>
-      <c r="E45" s="5" t="s">
+      <c r="E45" t="s">
         <v>114</v>
       </c>
-      <c r="F45" s="5" t="s">
+      <c r="F45" t="s">
         <v>115</v>
       </c>
-      <c r="G45" s="5" t="s">
+      <c r="G45" t="s">
         <v>116</v>
       </c>
-      <c r="H45" s="7">
+      <c r="H45">
         <v>42578.632777777777</v>
       </c>
     </row>
-    <row r="46" spans="1:8">
-      <c r="A46" s="3">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A46">
         <v>4144897</v>
       </c>
-      <c r="B46" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C46" s="5" t="s">
+      <c r="B46" t="s">
+        <v>12</v>
+      </c>
+      <c r="C46" t="s">
         <v>17</v>
       </c>
-      <c r="D46" s="5">
+      <c r="D46">
         <v>11</v>
       </c>
-      <c r="E46" s="5" t="s">
+      <c r="E46" t="s">
         <v>117</v>
       </c>
-      <c r="F46" s="5" t="s">
+      <c r="F46" t="s">
         <v>118</v>
       </c>
-      <c r="G46" s="5" t="s">
+      <c r="G46" t="s">
         <v>20</v>
       </c>
-      <c r="H46" s="7">
+      <c r="H46">
         <v>42592.50439814815</v>
       </c>
     </row>
-    <row r="47" spans="1:8">
-      <c r="A47" s="3">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A47">
         <v>4153692</v>
       </c>
-      <c r="B47" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C47" s="5" t="s">
+      <c r="B47" t="s">
+        <v>12</v>
+      </c>
+      <c r="C47" t="s">
         <v>17</v>
       </c>
-      <c r="D47" s="5">
+      <c r="D47">
         <v>10</v>
       </c>
-      <c r="E47" s="5" t="s">
+      <c r="E47" t="s">
         <v>119</v>
       </c>
-      <c r="F47" s="5" t="s">
+      <c r="F47" t="s">
         <v>120</v>
       </c>
-      <c r="G47" s="5" t="s">
+      <c r="G47" t="s">
         <v>20</v>
       </c>
-      <c r="H47" s="7">
+      <c r="H47">
         <v>42578.621562499997</v>
       </c>
     </row>
-    <row r="48" spans="1:8">
-      <c r="A48" s="3">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A48">
         <v>4623081</v>
       </c>
-      <c r="B48" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C48" s="5" t="s">
+      <c r="B48" t="s">
+        <v>12</v>
+      </c>
+      <c r="C48" t="s">
         <v>17</v>
       </c>
-      <c r="D48" s="5">
+      <c r="D48">
         <v>20</v>
       </c>
-      <c r="E48" s="5" t="s">
+      <c r="E48" t="s">
         <v>121</v>
       </c>
-      <c r="F48" s="5" t="s">
+      <c r="F48" t="s">
         <v>122</v>
       </c>
-      <c r="G48" s="5" t="s">
+      <c r="G48" t="s">
         <v>20</v>
       </c>
-      <c r="H48" s="7">
+      <c r="H48">
         <v>42676.708240740743</v>
       </c>
     </row>
-    <row r="49" spans="1:8">
-      <c r="A49" s="3">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A49">
         <v>4639434</v>
       </c>
-      <c r="B49" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C49" s="5" t="s">
+      <c r="B49" t="s">
+        <v>12</v>
+      </c>
+      <c r="C49" t="s">
         <v>17</v>
       </c>
-      <c r="D49" s="5">
+      <c r="D49">
         <v>5</v>
       </c>
-      <c r="E49" s="5" t="s">
+      <c r="E49" t="s">
         <v>123</v>
       </c>
-      <c r="F49" s="5" t="s">
+      <c r="F49" t="s">
         <v>124</v>
       </c>
-      <c r="G49" s="5" t="s">
+      <c r="G49" t="s">
         <v>59</v>
       </c>
-      <c r="H49" s="7">
+      <c r="H49">
         <v>42676.708240740743</v>
       </c>
     </row>
-    <row r="50" spans="1:8">
-      <c r="A50" s="8">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A50">
         <v>4647242</v>
       </c>
-      <c r="B50" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="C50" s="9" t="s">
+      <c r="B50" t="s">
+        <v>12</v>
+      </c>
+      <c r="C50" t="s">
         <v>17</v>
       </c>
-      <c r="D50" s="9">
+      <c r="D50">
         <v>15</v>
       </c>
-      <c r="E50" s="9" t="s">
+      <c r="E50" t="s">
         <v>125</v>
       </c>
-      <c r="F50" s="9" t="s">
+      <c r="F50" t="s">
         <v>126</v>
       </c>
-      <c r="G50" s="9" t="s">
+      <c r="G50" t="s">
         <v>20</v>
       </c>
-      <c r="H50" s="10">
+      <c r="H50">
         <v>42676.708240740743</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A1:A1048576">
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
-  </conditionalFormatting>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -3493,37 +3410,37 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E60F5AD9-1DF0-4940-8654-9F3C44B80CE7}">
   <dimension ref="B2:B7"/>
-  <sheetFormatPr defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="20.69921875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:2" ht="17.399999999999999">
+    <row r="2" spans="2:2" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="B2" s="1" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="3" spans="2:2" ht="16.8">
+    <row r="3" spans="2:2" ht="16.8" x14ac:dyDescent="0.25">
       <c r="B3" s="2" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="4" spans="2:2" ht="16.8">
+    <row r="4" spans="2:2" ht="16.8" x14ac:dyDescent="0.25">
       <c r="B4" s="2" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="5" spans="2:2" ht="16.8">
+    <row r="5" spans="2:2" ht="16.8" x14ac:dyDescent="0.25">
       <c r="B5" s="2" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="6" spans="2:2" ht="16.8">
+    <row r="6" spans="2:2" ht="16.8" x14ac:dyDescent="0.25">
       <c r="B6" s="2" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="7" spans="2:2" ht="16.8">
+    <row r="7" spans="2:2" ht="16.8" x14ac:dyDescent="0.25">
       <c r="B7" s="2" t="s">
         <v>132</v>
       </c>
@@ -3847,15 +3764,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
@@ -3873,6 +3781,15 @@
     <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3897,14 +3814,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C91CA977-A602-44A9-8850-357798C720DC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E1F5EDDD-2981-4B65-B7EF-62D15E153F33}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -3916,6 +3825,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C91CA977-A602-44A9-8850-357798C720DC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata"/>
 </file>
</xml_diff>

<commit_message>
upload dashboard tutorial solution and wk5 slides
</commit_message>
<xml_diff>
--- a/wk4/Tree Inventory Data Exercise.xlsx
+++ b/wk4/Tree Inventory Data Exercise.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Laptop W11\working_folder\Personales\Upright\Data_Science\instructor-dab-sep-2026\wk4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27936A55-3514-4B47-A771-6EEED62ACD6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{127AEA2D-3099-4332-8300-9B0D9A19C842}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{422E36C7-441B-4CF8-9E4B-F37F4293F8CF}"/>
   </bookViews>
@@ -520,17 +520,7 @@
     <cellStyle name="Heading 1 2" xfId="1" xr:uid="{78F2CDC0-5A06-4236-BE4B-C8FFA046B446}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="3">
     <dxf>
       <font>
         <b/>
@@ -594,9 +584,9 @@
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="TableStyleLight6 2" pivot="0" count="3" xr9:uid="{7A2670F4-CCC3-8044-96E0-9D071E21DDAD}">
-      <tableStyleElement type="wholeTable" dxfId="3"/>
-      <tableStyleElement type="headerRow" dxfId="2"/>
-      <tableStyleElement type="totalRow" dxfId="1"/>
+      <tableStyleElement type="wholeTable" dxfId="2"/>
+      <tableStyleElement type="headerRow" dxfId="1"/>
+      <tableStyleElement type="totalRow" dxfId="0"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -2099,10 +2089,10 @@
   <dimension ref="A1:H50"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.09765625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.3984375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.69921875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.8984375" customWidth="1"/>
+    <col min="2" max="2" width="12.09765625" customWidth="1"/>
+    <col min="3" max="3" width="12.8984375" customWidth="1"/>
+    <col min="4" max="4" width="17.8984375" customWidth="1"/>
     <col min="5" max="5" width="28.19921875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="31.5" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="22.3984375" bestFit="1" customWidth="1"/>
@@ -3764,6 +3754,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
@@ -3781,15 +3780,6 @@
     <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3814,6 +3804,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C91CA977-A602-44A9-8850-357798C720DC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E1F5EDDD-2981-4B65-B7EF-62D15E153F33}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -3825,14 +3823,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C91CA977-A602-44A9-8850-357798C720DC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata"/>
 </file>
</xml_diff>